<commit_message>
Actualizacion y mejoras en la estructura de la base de datos y en la interfaz de usuario para la gestión de inventario. Se han agregado nuevos diálogos para la importación de existencias, manejo de monedas y visualización preliminar de datos. Además, se han realizado ajustes en los scripts de generación de PDF e importación de transacciones para mejorar la funcionalidad y la experiencia del usuario.
</commit_message>
<xml_diff>
--- a/Docs/Estructura DB/Integracion Estructura DBIsam  -  SQLite SoperacionInv-01Qw.xlsx
+++ b/Docs/Estructura DB/Integracion Estructura DBIsam  -  SQLite SoperacionInv-01Qw.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Desarrollos\MyPython\Tkinter\ArkConInv\Docs\Estructura DB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568EF23A-A8CD-47A2-B84A-DDEF262B06C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA3F5CEB-273B-4EEF-A1A5-DB11D6E4DB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Integracion Estructura DBIsam  " sheetId="1" r:id="rId1"/>
     <sheet name="Integracion Estructura SQLite" sheetId="2" r:id="rId2"/>
+    <sheet name="Estructura Existencia" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1539" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1614" uniqueCount="411">
   <si>
     <t>Destination Inventory Table Structure ark_transacciones</t>
   </si>
@@ -1127,6 +1128,147 @@
   </si>
   <si>
     <t>trn_UserLastUpdate</t>
+  </si>
+  <si>
+    <t>Source Inventory Table Structure SinvDep No Homologado</t>
+  </si>
+  <si>
+    <t>FT_TIPO</t>
+  </si>
+  <si>
+    <t>SMALLINT NOT NULL</t>
+  </si>
+  <si>
+    <t>FT_CODIGOPRODUCTO</t>
+  </si>
+  <si>
+    <t>FT_CODIGODEPOSITO</t>
+  </si>
+  <si>
+    <t>FT_LOTE</t>
+  </si>
+  <si>
+    <t>FT_LOTEAUTOINCREMENT</t>
+  </si>
+  <si>
+    <t>FT_NOLINEA</t>
+  </si>
+  <si>
+    <t>FT_STATUS</t>
+  </si>
+  <si>
+    <t>FT_PUESTO</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIA</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIADETALLADA</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIAAPARTADA</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIAORDENCOMPRA</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIAPEDIDO</t>
+  </si>
+  <si>
+    <t>FT_INVENTARIOINICIALBS</t>
+  </si>
+  <si>
+    <t>FT_INVENTARIOINICIALBSCIERRE</t>
+  </si>
+  <si>
+    <t>FT_INVENTARIOINICIALUND</t>
+  </si>
+  <si>
+    <t>FT_INVENTARIOINICIALCIERRE</t>
+  </si>
+  <si>
+    <t>FT_CTDTRANSITO</t>
+  </si>
+  <si>
+    <t>FT_VISIBLE</t>
+  </si>
+  <si>
+    <t>FT_CODEBARRA</t>
+  </si>
+  <si>
+    <t>FT_EXISTENCIAAJUSTE</t>
+  </si>
+  <si>
+    <t>FT_CODE</t>
+  </si>
+  <si>
+    <t>Destination Inventory Table Structure ark_existencia_actual</t>
+  </si>
+  <si>
+    <t>exa_tipo</t>
+  </si>
+  <si>
+    <t>exa_codigoproducto</t>
+  </si>
+  <si>
+    <t>exa_codigodeposito</t>
+  </si>
+  <si>
+    <t>exa_lote</t>
+  </si>
+  <si>
+    <t>exa_loteautoincrement</t>
+  </si>
+  <si>
+    <t>exa_nolinea</t>
+  </si>
+  <si>
+    <t>exa_status</t>
+  </si>
+  <si>
+    <t>exa_puesto</t>
+  </si>
+  <si>
+    <t>exa_existencia</t>
+  </si>
+  <si>
+    <t>exa_existenciadetallada</t>
+  </si>
+  <si>
+    <t>exa_existenciaapartada</t>
+  </si>
+  <si>
+    <t>exa_existenciaordencompra</t>
+  </si>
+  <si>
+    <t>exa_existenciapedido</t>
+  </si>
+  <si>
+    <t>exa_inventarioinicialbs</t>
+  </si>
+  <si>
+    <t>exa_inventarioinicialbscierre</t>
+  </si>
+  <si>
+    <t>exa_inventarioinicialund</t>
+  </si>
+  <si>
+    <t>exa_inventarioinicialcierre</t>
+  </si>
+  <si>
+    <t>exa_ctdtransito</t>
+  </si>
+  <si>
+    <t>exa_visible</t>
+  </si>
+  <si>
+    <t>exa_codebarra</t>
+  </si>
+  <si>
+    <t>exa_existenciaajuste</t>
+  </si>
+  <si>
+    <t>exa_code</t>
   </si>
 </sst>
 </file>
@@ -1645,7 +1787,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1666,9 +1808,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1676,6 +1815,10 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="37" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Énfasis1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -2040,18 +2183,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8" t="s">
+      <c r="B1" s="11"/>
+      <c r="C1" s="11" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8" t="s">
+      <c r="D1" s="11"/>
+      <c r="E1" s="11" t="s">
         <v>333</v>
       </c>
-      <c r="F1" s="8"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6">
       <c r="A2" t="s">
@@ -4621,7 +4764,7 @@
       <c r="B2" t="s">
         <v>322</v>
       </c>
-      <c r="C2" s="9" t="s">
+      <c r="C2" s="8" t="s">
         <v>322</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -4641,7 +4784,7 @@
       <c r="B3" t="s">
         <v>338</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>338</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -4661,7 +4804,7 @@
       <c r="B4" t="s">
         <v>323</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>323</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -4681,7 +4824,7 @@
       <c r="B5" t="s">
         <v>324</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="8" t="s">
         <v>324</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -4701,7 +4844,7 @@
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="8" t="s">
         <v>5</v>
       </c>
       <c r="D6" s="1">
@@ -4713,7 +4856,7 @@
       <c r="G6" t="s">
         <v>353</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="H6" s="8" t="s">
         <v>3</v>
       </c>
       <c r="I6" t="str">
@@ -4728,7 +4871,7 @@
       <c r="B7" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="9" t="s">
+      <c r="C7" s="8" t="s">
         <v>9</v>
       </c>
       <c r="D7" s="1">
@@ -4741,7 +4884,7 @@
       <c r="G7" t="s">
         <v>353</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="H7" s="8" t="s">
         <v>7</v>
       </c>
       <c r="I7" t="str">
@@ -4756,7 +4899,7 @@
       <c r="B8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="9" t="s">
+      <c r="C8" s="8" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="6">
@@ -4769,7 +4912,7 @@
       <c r="G8" t="s">
         <v>353</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="8" t="s">
         <v>11</v>
       </c>
       <c r="I8" t="str">
@@ -4784,7 +4927,7 @@
       <c r="B9" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="9" t="s">
+      <c r="C9" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D9" s="6">
@@ -4797,7 +4940,7 @@
       <c r="G9" t="s">
         <v>353</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="H9" s="8" t="s">
         <v>15</v>
       </c>
       <c r="I9" t="str">
@@ -4812,7 +4955,7 @@
       <c r="B10" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="9" t="s">
+      <c r="C10" s="8" t="s">
         <v>21</v>
       </c>
       <c r="D10" s="6">
@@ -4825,7 +4968,7 @@
       <c r="G10" t="s">
         <v>353</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="H10" s="8" t="s">
         <v>19</v>
       </c>
       <c r="I10" t="str">
@@ -4840,7 +4983,7 @@
       <c r="B11" t="s">
         <v>24</v>
       </c>
-      <c r="C11" s="9" t="s">
+      <c r="C11" s="8" t="s">
         <v>24</v>
       </c>
       <c r="D11" s="6">
@@ -4853,7 +4996,7 @@
       <c r="G11" t="s">
         <v>353</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="H11" s="8" t="s">
         <v>22</v>
       </c>
       <c r="I11" t="str">
@@ -4868,7 +5011,7 @@
       <c r="B12" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="8" t="s">
         <v>27</v>
       </c>
       <c r="D12" s="6">
@@ -4881,7 +5024,7 @@
       <c r="G12" t="s">
         <v>353</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="8" t="s">
         <v>26</v>
       </c>
       <c r="I12" t="str">
@@ -4896,7 +5039,7 @@
       <c r="B13" t="s">
         <v>29</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C13" s="8" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="6">
@@ -4909,7 +5052,7 @@
       <c r="G13" t="s">
         <v>353</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="H13" s="8" t="s">
         <v>28</v>
       </c>
       <c r="I13" t="str">
@@ -4924,7 +5067,7 @@
       <c r="B14" t="s">
         <v>31</v>
       </c>
-      <c r="C14" s="9" t="s">
+      <c r="C14" s="8" t="s">
         <v>31</v>
       </c>
       <c r="D14" s="6">
@@ -4937,7 +5080,7 @@
       <c r="G14" t="s">
         <v>353</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="H14" s="8" t="s">
         <v>30</v>
       </c>
       <c r="I14" t="str">
@@ -4952,7 +5095,7 @@
       <c r="B15" t="s">
         <v>33</v>
       </c>
-      <c r="C15" s="9" t="s">
+      <c r="C15" s="8" t="s">
         <v>33</v>
       </c>
       <c r="D15" s="6">
@@ -4965,7 +5108,7 @@
       <c r="G15" t="s">
         <v>353</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="H15" s="8" t="s">
         <v>32</v>
       </c>
       <c r="I15" t="str">
@@ -4980,7 +5123,7 @@
       <c r="B16" t="s">
         <v>35</v>
       </c>
-      <c r="C16" s="9" t="s">
+      <c r="C16" s="8" t="s">
         <v>35</v>
       </c>
       <c r="D16" s="6">
@@ -4993,7 +5136,7 @@
       <c r="G16" t="s">
         <v>353</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="8" t="s">
         <v>34</v>
       </c>
       <c r="I16" t="str">
@@ -5008,7 +5151,7 @@
       <c r="B17" t="s">
         <v>38</v>
       </c>
-      <c r="C17" s="9" t="s">
+      <c r="C17" s="8" t="s">
         <v>38</v>
       </c>
       <c r="D17" s="6">
@@ -5021,7 +5164,7 @@
       <c r="G17" t="s">
         <v>353</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="H17" s="8" t="s">
         <v>36</v>
       </c>
       <c r="I17" t="str">
@@ -5036,7 +5179,7 @@
       <c r="B18" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="9" t="s">
+      <c r="C18" s="8" t="s">
         <v>41</v>
       </c>
       <c r="D18" s="6">
@@ -5049,7 +5192,7 @@
       <c r="G18" t="s">
         <v>353</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="H18" s="8" t="s">
         <v>40</v>
       </c>
       <c r="I18" t="str">
@@ -5064,7 +5207,7 @@
       <c r="B19" t="s">
         <v>43</v>
       </c>
-      <c r="C19" s="9" t="s">
+      <c r="C19" s="8" t="s">
         <v>43</v>
       </c>
       <c r="D19" s="6">
@@ -5077,7 +5220,7 @@
       <c r="G19" t="s">
         <v>353</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="H19" s="8" t="s">
         <v>42</v>
       </c>
       <c r="I19" t="str">
@@ -5092,7 +5235,7 @@
       <c r="B20" t="s">
         <v>45</v>
       </c>
-      <c r="C20" s="9" t="s">
+      <c r="C20" s="8" t="s">
         <v>45</v>
       </c>
       <c r="D20" s="6">
@@ -5105,7 +5248,7 @@
       <c r="G20" t="s">
         <v>353</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="8" t="s">
         <v>44</v>
       </c>
       <c r="I20" t="str">
@@ -5120,7 +5263,7 @@
       <c r="B21" t="s">
         <v>48</v>
       </c>
-      <c r="C21" s="9" t="s">
+      <c r="C21" s="8" t="s">
         <v>48</v>
       </c>
       <c r="D21" s="6">
@@ -5133,7 +5276,7 @@
       <c r="G21" t="s">
         <v>353</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="H21" s="8" t="s">
         <v>46</v>
       </c>
       <c r="I21" t="str">
@@ -5148,7 +5291,7 @@
       <c r="B22" t="s">
         <v>50</v>
       </c>
-      <c r="C22" s="9" t="s">
+      <c r="C22" s="8" t="s">
         <v>50</v>
       </c>
       <c r="D22" s="6">
@@ -5161,7 +5304,7 @@
       <c r="G22" t="s">
         <v>353</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="H22" s="8" t="s">
         <v>49</v>
       </c>
       <c r="I22" t="str">
@@ -5176,7 +5319,7 @@
       <c r="B23" t="s">
         <v>53</v>
       </c>
-      <c r="C23" s="9" t="s">
+      <c r="C23" s="8" t="s">
         <v>53</v>
       </c>
       <c r="D23" s="6">
@@ -5189,7 +5332,7 @@
       <c r="G23" t="s">
         <v>353</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="H23" s="8" t="s">
         <v>51</v>
       </c>
       <c r="I23" t="str">
@@ -5204,7 +5347,7 @@
       <c r="B24" t="s">
         <v>56</v>
       </c>
-      <c r="C24" s="9" t="s">
+      <c r="C24" s="8" t="s">
         <v>56</v>
       </c>
       <c r="D24" s="6">
@@ -5217,7 +5360,7 @@
       <c r="G24" t="s">
         <v>353</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="H24" s="8" t="s">
         <v>54</v>
       </c>
       <c r="I24" t="str">
@@ -5232,7 +5375,7 @@
       <c r="B25" t="s">
         <v>58</v>
       </c>
-      <c r="C25" s="9" t="s">
+      <c r="C25" s="8" t="s">
         <v>58</v>
       </c>
       <c r="D25" s="6">
@@ -5245,7 +5388,7 @@
       <c r="G25" t="s">
         <v>353</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="H25" s="8" t="s">
         <v>57</v>
       </c>
       <c r="I25" t="str">
@@ -5260,7 +5403,7 @@
       <c r="B26" t="s">
         <v>61</v>
       </c>
-      <c r="C26" s="9" t="s">
+      <c r="C26" s="8" t="s">
         <v>61</v>
       </c>
       <c r="D26" s="6">
@@ -5273,7 +5416,7 @@
       <c r="G26" t="s">
         <v>353</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="H26" s="8" t="s">
         <v>59</v>
       </c>
       <c r="I26" t="str">
@@ -5288,7 +5431,7 @@
       <c r="B27" t="s">
         <v>63</v>
       </c>
-      <c r="C27" s="9" t="s">
+      <c r="C27" s="8" t="s">
         <v>63</v>
       </c>
       <c r="D27" s="6">
@@ -5301,7 +5444,7 @@
       <c r="G27" t="s">
         <v>353</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="H27" s="8" t="s">
         <v>62</v>
       </c>
       <c r="I27" t="str">
@@ -5316,7 +5459,7 @@
       <c r="B28" t="s">
         <v>65</v>
       </c>
-      <c r="C28" s="9" t="s">
+      <c r="C28" s="8" t="s">
         <v>65</v>
       </c>
       <c r="D28" s="6">
@@ -5329,7 +5472,7 @@
       <c r="G28" t="s">
         <v>353</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="H28" s="8" t="s">
         <v>64</v>
       </c>
       <c r="I28" t="str">
@@ -5344,7 +5487,7 @@
       <c r="B29" t="s">
         <v>67</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="8" t="s">
         <v>67</v>
       </c>
       <c r="D29" s="6">
@@ -5357,7 +5500,7 @@
       <c r="G29" t="s">
         <v>353</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="H29" s="8" t="s">
         <v>66</v>
       </c>
       <c r="I29" t="str">
@@ -5372,7 +5515,7 @@
       <c r="B30" t="s">
         <v>69</v>
       </c>
-      <c r="C30" s="9" t="s">
+      <c r="C30" s="8" t="s">
         <v>69</v>
       </c>
       <c r="D30" s="6">
@@ -5385,7 +5528,7 @@
       <c r="G30" t="s">
         <v>353</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="H30" s="8" t="s">
         <v>68</v>
       </c>
       <c r="I30" t="str">
@@ -5400,7 +5543,7 @@
       <c r="B31" t="s">
         <v>71</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="8" t="s">
         <v>71</v>
       </c>
       <c r="D31" s="6">
@@ -5413,7 +5556,7 @@
       <c r="G31" t="s">
         <v>353</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="H31" s="8" t="s">
         <v>70</v>
       </c>
       <c r="I31" t="str">
@@ -5428,7 +5571,7 @@
       <c r="B32" t="s">
         <v>74</v>
       </c>
-      <c r="C32" s="9" t="s">
+      <c r="C32" s="8" t="s">
         <v>74</v>
       </c>
       <c r="D32" s="6">
@@ -5441,7 +5584,7 @@
       <c r="G32" t="s">
         <v>353</v>
       </c>
-      <c r="H32" s="9" t="s">
+      <c r="H32" s="8" t="s">
         <v>72</v>
       </c>
       <c r="I32" t="str">
@@ -5456,7 +5599,7 @@
       <c r="B33" t="s">
         <v>76</v>
       </c>
-      <c r="C33" s="9" t="s">
+      <c r="C33" s="8" t="s">
         <v>76</v>
       </c>
       <c r="D33" s="6">
@@ -5469,7 +5612,7 @@
       <c r="G33" t="s">
         <v>353</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="H33" s="8" t="s">
         <v>75</v>
       </c>
       <c r="I33" t="str">
@@ -5484,7 +5627,7 @@
       <c r="B34" t="s">
         <v>78</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="8" t="s">
         <v>78</v>
       </c>
       <c r="D34" s="6">
@@ -5497,7 +5640,7 @@
       <c r="G34" t="s">
         <v>353</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="H34" s="8" t="s">
         <v>77</v>
       </c>
       <c r="I34" t="str">
@@ -5512,7 +5655,7 @@
       <c r="B35" t="s">
         <v>80</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="8" t="s">
         <v>80</v>
       </c>
       <c r="D35" s="6">
@@ -5525,7 +5668,7 @@
       <c r="G35" t="s">
         <v>353</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="H35" s="8" t="s">
         <v>79</v>
       </c>
       <c r="I35" t="str">
@@ -5540,7 +5683,7 @@
       <c r="B36" t="s">
         <v>82</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="C36" s="8" t="s">
         <v>82</v>
       </c>
       <c r="D36" s="6">
@@ -5553,7 +5696,7 @@
       <c r="G36" t="s">
         <v>353</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="H36" s="8" t="s">
         <v>81</v>
       </c>
       <c r="I36" t="str">
@@ -5568,7 +5711,7 @@
       <c r="B37" t="s">
         <v>84</v>
       </c>
-      <c r="C37" s="9" t="s">
+      <c r="C37" s="8" t="s">
         <v>84</v>
       </c>
       <c r="D37" s="6">
@@ -5581,7 +5724,7 @@
       <c r="G37" t="s">
         <v>353</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="H37" s="8" t="s">
         <v>83</v>
       </c>
       <c r="I37" t="str">
@@ -5596,7 +5739,7 @@
       <c r="B38" t="s">
         <v>86</v>
       </c>
-      <c r="C38" s="9" t="s">
+      <c r="C38" s="8" t="s">
         <v>86</v>
       </c>
       <c r="D38" s="6">
@@ -5609,7 +5752,7 @@
       <c r="G38" t="s">
         <v>353</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="H38" s="8" t="s">
         <v>85</v>
       </c>
       <c r="I38" t="str">
@@ -5624,7 +5767,7 @@
       <c r="B39" t="s">
         <v>88</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="C39" s="8" t="s">
         <v>88</v>
       </c>
       <c r="D39" s="6">
@@ -5637,7 +5780,7 @@
       <c r="G39" t="s">
         <v>353</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="H39" s="8" t="s">
         <v>87</v>
       </c>
       <c r="I39" t="str">
@@ -5652,7 +5795,7 @@
       <c r="B40" t="s">
         <v>90</v>
       </c>
-      <c r="C40" s="9" t="s">
+      <c r="C40" s="8" t="s">
         <v>90</v>
       </c>
       <c r="D40" s="6">
@@ -5665,7 +5808,7 @@
       <c r="G40" t="s">
         <v>353</v>
       </c>
-      <c r="H40" s="9" t="s">
+      <c r="H40" s="8" t="s">
         <v>89</v>
       </c>
       <c r="I40" t="str">
@@ -5680,7 +5823,7 @@
       <c r="B41" t="s">
         <v>92</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="8" t="s">
         <v>92</v>
       </c>
       <c r="D41" s="6">
@@ -5693,7 +5836,7 @@
       <c r="G41" t="s">
         <v>353</v>
       </c>
-      <c r="H41" s="9" t="s">
+      <c r="H41" s="8" t="s">
         <v>91</v>
       </c>
       <c r="I41" t="str">
@@ -5708,7 +5851,7 @@
       <c r="B42" t="s">
         <v>94</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="8" t="s">
         <v>94</v>
       </c>
       <c r="D42" s="6">
@@ -5721,7 +5864,7 @@
       <c r="G42" t="s">
         <v>353</v>
       </c>
-      <c r="H42" s="9" t="s">
+      <c r="H42" s="8" t="s">
         <v>93</v>
       </c>
       <c r="I42" t="str">
@@ -5736,7 +5879,7 @@
       <c r="B43" t="s">
         <v>96</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="8" t="s">
         <v>96</v>
       </c>
       <c r="D43" s="6">
@@ -5749,7 +5892,7 @@
       <c r="G43" t="s">
         <v>353</v>
       </c>
-      <c r="H43" s="9" t="s">
+      <c r="H43" s="8" t="s">
         <v>95</v>
       </c>
       <c r="I43" t="str">
@@ -5764,7 +5907,7 @@
       <c r="B44" t="s">
         <v>98</v>
       </c>
-      <c r="C44" s="9" t="s">
+      <c r="C44" s="8" t="s">
         <v>98</v>
       </c>
       <c r="D44" s="6">
@@ -5777,7 +5920,7 @@
       <c r="G44" t="s">
         <v>353</v>
       </c>
-      <c r="H44" s="9" t="s">
+      <c r="H44" s="8" t="s">
         <v>97</v>
       </c>
       <c r="I44" t="str">
@@ -5792,7 +5935,7 @@
       <c r="B45" t="s">
         <v>100</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="8" t="s">
         <v>100</v>
       </c>
       <c r="D45" s="6">
@@ -5805,7 +5948,7 @@
       <c r="G45" t="s">
         <v>353</v>
       </c>
-      <c r="H45" s="9" t="s">
+      <c r="H45" s="8" t="s">
         <v>99</v>
       </c>
       <c r="I45" t="str">
@@ -5820,7 +5963,7 @@
       <c r="B46" t="s">
         <v>102</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="8" t="s">
         <v>102</v>
       </c>
       <c r="D46" s="6">
@@ -5833,7 +5976,7 @@
       <c r="G46" t="s">
         <v>353</v>
       </c>
-      <c r="H46" s="9" t="s">
+      <c r="H46" s="8" t="s">
         <v>101</v>
       </c>
       <c r="I46" t="str">
@@ -5848,7 +5991,7 @@
       <c r="B47" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="9" t="s">
+      <c r="C47" s="8" t="s">
         <v>104</v>
       </c>
       <c r="D47" s="6">
@@ -5861,7 +6004,7 @@
       <c r="G47" t="s">
         <v>353</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="H47" s="8" t="s">
         <v>103</v>
       </c>
       <c r="I47" t="str">
@@ -5876,7 +6019,7 @@
       <c r="B48" t="s">
         <v>107</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="8" t="s">
         <v>107</v>
       </c>
       <c r="D48" s="6">
@@ -5889,7 +6032,7 @@
       <c r="G48" t="s">
         <v>353</v>
       </c>
-      <c r="H48" s="9" t="s">
+      <c r="H48" s="8" t="s">
         <v>105</v>
       </c>
       <c r="I48" t="str">
@@ -5904,7 +6047,7 @@
       <c r="B49" t="s">
         <v>109</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="8" t="s">
         <v>109</v>
       </c>
       <c r="D49" s="6">
@@ -5917,7 +6060,7 @@
       <c r="G49" t="s">
         <v>353</v>
       </c>
-      <c r="H49" s="9" t="s">
+      <c r="H49" s="8" t="s">
         <v>108</v>
       </c>
       <c r="I49" t="str">
@@ -5932,7 +6075,7 @@
       <c r="B50" t="s">
         <v>111</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="8" t="s">
         <v>111</v>
       </c>
       <c r="D50" s="6">
@@ -5945,7 +6088,7 @@
       <c r="G50" t="s">
         <v>353</v>
       </c>
-      <c r="H50" s="9" t="s">
+      <c r="H50" s="8" t="s">
         <v>110</v>
       </c>
       <c r="I50" t="str">
@@ -5960,7 +6103,7 @@
       <c r="B51" t="s">
         <v>113</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="8" t="s">
         <v>113</v>
       </c>
       <c r="D51" s="6">
@@ -5973,7 +6116,7 @@
       <c r="G51" t="s">
         <v>353</v>
       </c>
-      <c r="H51" s="9" t="s">
+      <c r="H51" s="8" t="s">
         <v>112</v>
       </c>
       <c r="I51" t="str">
@@ -5988,7 +6131,7 @@
       <c r="B52" t="s">
         <v>115</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="8" t="s">
         <v>115</v>
       </c>
       <c r="D52" s="6">
@@ -6001,7 +6144,7 @@
       <c r="G52" t="s">
         <v>353</v>
       </c>
-      <c r="H52" s="9" t="s">
+      <c r="H52" s="8" t="s">
         <v>114</v>
       </c>
       <c r="I52" t="str">
@@ -6016,7 +6159,7 @@
       <c r="B53" t="s">
         <v>117</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="8" t="s">
         <v>117</v>
       </c>
       <c r="D53" s="6">
@@ -6029,7 +6172,7 @@
       <c r="G53" t="s">
         <v>353</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="H53" s="8" t="s">
         <v>116</v>
       </c>
       <c r="I53" t="str">
@@ -6044,7 +6187,7 @@
       <c r="B54" t="s">
         <v>119</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="8" t="s">
         <v>119</v>
       </c>
       <c r="D54" s="6">
@@ -6057,7 +6200,7 @@
       <c r="G54" t="s">
         <v>353</v>
       </c>
-      <c r="H54" s="9" t="s">
+      <c r="H54" s="8" t="s">
         <v>118</v>
       </c>
       <c r="I54" t="str">
@@ -6072,7 +6215,7 @@
       <c r="B55" t="s">
         <v>121</v>
       </c>
-      <c r="C55" s="9" t="s">
+      <c r="C55" s="8" t="s">
         <v>121</v>
       </c>
       <c r="D55" s="6">
@@ -6085,7 +6228,7 @@
       <c r="G55" t="s">
         <v>353</v>
       </c>
-      <c r="H55" s="9" t="s">
+      <c r="H55" s="8" t="s">
         <v>120</v>
       </c>
       <c r="I55" t="str">
@@ -6100,7 +6243,7 @@
       <c r="B56" t="s">
         <v>123</v>
       </c>
-      <c r="C56" s="9" t="s">
+      <c r="C56" s="8" t="s">
         <v>123</v>
       </c>
       <c r="D56" s="6">
@@ -6113,7 +6256,7 @@
       <c r="G56" t="s">
         <v>353</v>
       </c>
-      <c r="H56" s="9" t="s">
+      <c r="H56" s="8" t="s">
         <v>122</v>
       </c>
       <c r="I56" t="str">
@@ -6141,10 +6284,10 @@
       <c r="G57" t="s">
         <v>353</v>
       </c>
-      <c r="H57" s="10" t="s">
+      <c r="H57" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="I57" s="11" t="str">
+      <c r="I57" s="10" t="str">
         <f t="shared" si="0"/>
         <v>Si</v>
       </c>
@@ -6156,7 +6299,7 @@
       <c r="B58" t="s">
         <v>128</v>
       </c>
-      <c r="C58" s="9" t="s">
+      <c r="C58" s="8" t="s">
         <v>128</v>
       </c>
       <c r="D58" s="6">
@@ -6169,7 +6312,7 @@
       <c r="G58" t="s">
         <v>353</v>
       </c>
-      <c r="H58" s="9" t="s">
+      <c r="H58" s="8" t="s">
         <v>127</v>
       </c>
       <c r="I58" t="str">
@@ -6184,7 +6327,7 @@
       <c r="B59" t="s">
         <v>130</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="C59" s="8" t="s">
         <v>130</v>
       </c>
       <c r="D59" s="6">
@@ -6197,7 +6340,7 @@
       <c r="G59" t="s">
         <v>353</v>
       </c>
-      <c r="H59" s="9" t="s">
+      <c r="H59" s="8" t="s">
         <v>129</v>
       </c>
       <c r="I59" t="str">
@@ -6212,7 +6355,7 @@
       <c r="B60" t="s">
         <v>132</v>
       </c>
-      <c r="C60" s="9" t="s">
+      <c r="C60" s="8" t="s">
         <v>132</v>
       </c>
       <c r="D60" s="6">
@@ -6225,7 +6368,7 @@
       <c r="G60" t="s">
         <v>353</v>
       </c>
-      <c r="H60" s="9" t="s">
+      <c r="H60" s="8" t="s">
         <v>131</v>
       </c>
       <c r="I60" t="str">
@@ -6240,7 +6383,7 @@
       <c r="B61" t="s">
         <v>134</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C61" s="8" t="s">
         <v>134</v>
       </c>
       <c r="D61" s="6">
@@ -6253,7 +6396,7 @@
       <c r="G61" t="s">
         <v>353</v>
       </c>
-      <c r="H61" s="9" t="s">
+      <c r="H61" s="8" t="s">
         <v>133</v>
       </c>
       <c r="I61" t="str">
@@ -6281,10 +6424,10 @@
       <c r="G62" t="s">
         <v>353</v>
       </c>
-      <c r="H62" s="10" t="s">
+      <c r="H62" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="I62" s="11" t="str">
+      <c r="I62" s="10" t="str">
         <f t="shared" si="0"/>
         <v>Si</v>
       </c>
@@ -6296,7 +6439,7 @@
       <c r="B63" t="s">
         <v>138</v>
       </c>
-      <c r="C63" s="9" t="s">
+      <c r="C63" s="8" t="s">
         <v>138</v>
       </c>
       <c r="D63" s="6">
@@ -6309,7 +6452,7 @@
       <c r="G63" t="s">
         <v>353</v>
       </c>
-      <c r="H63" s="9" t="s">
+      <c r="H63" s="8" t="s">
         <v>137</v>
       </c>
       <c r="I63" t="str">
@@ -6324,7 +6467,7 @@
       <c r="B64" t="s">
         <v>140</v>
       </c>
-      <c r="C64" s="9" t="s">
+      <c r="C64" s="8" t="s">
         <v>140</v>
       </c>
       <c r="D64" s="6">
@@ -6337,7 +6480,7 @@
       <c r="G64" t="s">
         <v>353</v>
       </c>
-      <c r="H64" s="9" t="s">
+      <c r="H64" s="8" t="s">
         <v>139</v>
       </c>
       <c r="I64" t="str">
@@ -6352,7 +6495,7 @@
       <c r="B65" t="s">
         <v>142</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="8" t="s">
         <v>142</v>
       </c>
       <c r="D65" s="6">
@@ -6365,7 +6508,7 @@
       <c r="G65" t="s">
         <v>353</v>
       </c>
-      <c r="H65" s="9" t="s">
+      <c r="H65" s="8" t="s">
         <v>141</v>
       </c>
       <c r="I65" t="str">
@@ -6380,7 +6523,7 @@
       <c r="B66" t="s">
         <v>144</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="8" t="s">
         <v>144</v>
       </c>
       <c r="D66" s="6">
@@ -6393,7 +6536,7 @@
       <c r="G66" t="s">
         <v>353</v>
       </c>
-      <c r="H66" s="9" t="s">
+      <c r="H66" s="8" t="s">
         <v>143</v>
       </c>
       <c r="I66" t="str">
@@ -6408,7 +6551,7 @@
       <c r="B67" t="s">
         <v>146</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="8" t="s">
         <v>146</v>
       </c>
       <c r="D67" s="6">
@@ -6421,7 +6564,7 @@
       <c r="G67" t="s">
         <v>353</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H67" s="8" t="s">
         <v>145</v>
       </c>
       <c r="I67" t="str">
@@ -6436,7 +6579,7 @@
       <c r="B68" t="s">
         <v>148</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="C68" s="8" t="s">
         <v>148</v>
       </c>
       <c r="D68" s="6">
@@ -6449,7 +6592,7 @@
       <c r="G68" t="s">
         <v>353</v>
       </c>
-      <c r="H68" s="9" t="s">
+      <c r="H68" s="8" t="s">
         <v>147</v>
       </c>
       <c r="I68" t="str">
@@ -6464,7 +6607,7 @@
       <c r="B69" t="s">
         <v>151</v>
       </c>
-      <c r="C69" s="9" t="s">
+      <c r="C69" s="8" t="s">
         <v>151</v>
       </c>
       <c r="D69" s="6">
@@ -6477,7 +6620,7 @@
       <c r="G69" t="s">
         <v>353</v>
       </c>
-      <c r="H69" s="9" t="s">
+      <c r="H69" s="8" t="s">
         <v>149</v>
       </c>
       <c r="I69" t="str">
@@ -6492,7 +6635,7 @@
       <c r="B70" t="s">
         <v>153</v>
       </c>
-      <c r="C70" s="9" t="s">
+      <c r="C70" s="8" t="s">
         <v>153</v>
       </c>
       <c r="D70" s="6">
@@ -6505,7 +6648,7 @@
       <c r="G70" t="s">
         <v>353</v>
       </c>
-      <c r="H70" s="9" t="s">
+      <c r="H70" s="8" t="s">
         <v>152</v>
       </c>
       <c r="I70" t="str">
@@ -6520,7 +6663,7 @@
       <c r="B71" t="s">
         <v>155</v>
       </c>
-      <c r="C71" s="9" t="s">
+      <c r="C71" s="8" t="s">
         <v>155</v>
       </c>
       <c r="D71" s="6">
@@ -6533,7 +6676,7 @@
       <c r="G71" t="s">
         <v>353</v>
       </c>
-      <c r="H71" s="9" t="s">
+      <c r="H71" s="8" t="s">
         <v>154</v>
       </c>
       <c r="I71" t="str">
@@ -6548,7 +6691,7 @@
       <c r="B72" t="s">
         <v>158</v>
       </c>
-      <c r="C72" s="9" t="s">
+      <c r="C72" s="8" t="s">
         <v>158</v>
       </c>
       <c r="D72" s="6">
@@ -6561,7 +6704,7 @@
       <c r="G72" t="s">
         <v>353</v>
       </c>
-      <c r="H72" s="9" t="s">
+      <c r="H72" s="8" t="s">
         <v>156</v>
       </c>
       <c r="I72" t="str">
@@ -6576,7 +6719,7 @@
       <c r="B73" t="s">
         <v>160</v>
       </c>
-      <c r="C73" s="9" t="s">
+      <c r="C73" s="8" t="s">
         <v>160</v>
       </c>
       <c r="D73" s="6">
@@ -6589,7 +6732,7 @@
       <c r="G73" t="s">
         <v>353</v>
       </c>
-      <c r="H73" s="9" t="s">
+      <c r="H73" s="8" t="s">
         <v>159</v>
       </c>
       <c r="I73" t="str">
@@ -6604,7 +6747,7 @@
       <c r="B74" t="s">
         <v>162</v>
       </c>
-      <c r="C74" s="9" t="s">
+      <c r="C74" s="8" t="s">
         <v>162</v>
       </c>
       <c r="D74" s="6">
@@ -6617,7 +6760,7 @@
       <c r="G74" t="s">
         <v>353</v>
       </c>
-      <c r="H74" s="9" t="s">
+      <c r="H74" s="8" t="s">
         <v>161</v>
       </c>
       <c r="I74" t="str">
@@ -6632,7 +6775,7 @@
       <c r="B75" t="s">
         <v>164</v>
       </c>
-      <c r="C75" s="9" t="s">
+      <c r="C75" s="8" t="s">
         <v>164</v>
       </c>
       <c r="D75" s="6">
@@ -6645,7 +6788,7 @@
       <c r="G75" t="s">
         <v>353</v>
       </c>
-      <c r="H75" s="9" t="s">
+      <c r="H75" s="8" t="s">
         <v>163</v>
       </c>
       <c r="I75" t="str">
@@ -6660,7 +6803,7 @@
       <c r="B76" t="s">
         <v>166</v>
       </c>
-      <c r="C76" s="9" t="s">
+      <c r="C76" s="8" t="s">
         <v>166</v>
       </c>
       <c r="D76" s="6">
@@ -6673,7 +6816,7 @@
       <c r="G76" t="s">
         <v>353</v>
       </c>
-      <c r="H76" s="9" t="s">
+      <c r="H76" s="8" t="s">
         <v>165</v>
       </c>
       <c r="I76" t="str">
@@ -6688,7 +6831,7 @@
       <c r="B77" t="s">
         <v>169</v>
       </c>
-      <c r="C77" s="9" t="s">
+      <c r="C77" s="8" t="s">
         <v>169</v>
       </c>
       <c r="D77" s="6">
@@ -6701,7 +6844,7 @@
       <c r="G77" t="s">
         <v>353</v>
       </c>
-      <c r="H77" s="9" t="s">
+      <c r="H77" s="8" t="s">
         <v>167</v>
       </c>
       <c r="I77" t="str">
@@ -6716,7 +6859,7 @@
       <c r="B78" t="s">
         <v>171</v>
       </c>
-      <c r="C78" s="9" t="s">
+      <c r="C78" s="8" t="s">
         <v>171</v>
       </c>
       <c r="D78" s="6">
@@ -6729,7 +6872,7 @@
       <c r="G78" t="s">
         <v>353</v>
       </c>
-      <c r="H78" s="9" t="s">
+      <c r="H78" s="8" t="s">
         <v>170</v>
       </c>
       <c r="I78" t="str">
@@ -6744,7 +6887,7 @@
       <c r="B79" t="s">
         <v>173</v>
       </c>
-      <c r="C79" s="9" t="s">
+      <c r="C79" s="8" t="s">
         <v>173</v>
       </c>
       <c r="D79" s="6">
@@ -6757,7 +6900,7 @@
       <c r="G79" t="s">
         <v>353</v>
       </c>
-      <c r="H79" s="9" t="s">
+      <c r="H79" s="8" t="s">
         <v>172</v>
       </c>
       <c r="I79" t="str">
@@ -6772,7 +6915,7 @@
       <c r="B80" t="s">
         <v>175</v>
       </c>
-      <c r="C80" s="9" t="s">
+      <c r="C80" s="8" t="s">
         <v>175</v>
       </c>
       <c r="D80" s="6">
@@ -6785,7 +6928,7 @@
       <c r="G80" t="s">
         <v>353</v>
       </c>
-      <c r="H80" s="9" t="s">
+      <c r="H80" s="8" t="s">
         <v>174</v>
       </c>
       <c r="I80" t="str">
@@ -6800,7 +6943,7 @@
       <c r="B81" t="s">
         <v>177</v>
       </c>
-      <c r="C81" s="9" t="s">
+      <c r="C81" s="8" t="s">
         <v>177</v>
       </c>
       <c r="D81" s="6">
@@ -6813,7 +6956,7 @@
       <c r="G81" t="s">
         <v>353</v>
       </c>
-      <c r="H81" s="9" t="s">
+      <c r="H81" s="8" t="s">
         <v>176</v>
       </c>
       <c r="I81" t="str">
@@ -6828,7 +6971,7 @@
       <c r="B82" t="s">
         <v>179</v>
       </c>
-      <c r="C82" s="9" t="s">
+      <c r="C82" s="8" t="s">
         <v>179</v>
       </c>
       <c r="D82" s="6">
@@ -6841,7 +6984,7 @@
       <c r="G82" t="s">
         <v>353</v>
       </c>
-      <c r="H82" s="9" t="s">
+      <c r="H82" s="8" t="s">
         <v>178</v>
       </c>
       <c r="I82" t="str">
@@ -6856,7 +6999,7 @@
       <c r="B83" t="s">
         <v>181</v>
       </c>
-      <c r="C83" s="9" t="s">
+      <c r="C83" s="8" t="s">
         <v>181</v>
       </c>
       <c r="D83" s="6">
@@ -6869,7 +7012,7 @@
       <c r="G83" t="s">
         <v>353</v>
       </c>
-      <c r="H83" s="9" t="s">
+      <c r="H83" s="8" t="s">
         <v>180</v>
       </c>
       <c r="I83" t="str">
@@ -6884,7 +7027,7 @@
       <c r="B84" t="s">
         <v>183</v>
       </c>
-      <c r="C84" s="9" t="s">
+      <c r="C84" s="8" t="s">
         <v>183</v>
       </c>
       <c r="D84" s="6">
@@ -6897,7 +7040,7 @@
       <c r="G84" t="s">
         <v>353</v>
       </c>
-      <c r="H84" s="9" t="s">
+      <c r="H84" s="8" t="s">
         <v>182</v>
       </c>
       <c r="I84" t="str">
@@ -6912,7 +7055,7 @@
       <c r="B85" t="s">
         <v>185</v>
       </c>
-      <c r="C85" s="9" t="s">
+      <c r="C85" s="8" t="s">
         <v>185</v>
       </c>
       <c r="D85" s="6">
@@ -6925,7 +7068,7 @@
       <c r="G85" t="s">
         <v>353</v>
       </c>
-      <c r="H85" s="9" t="s">
+      <c r="H85" s="8" t="s">
         <v>184</v>
       </c>
       <c r="I85" t="str">
@@ -6940,7 +7083,7 @@
       <c r="B86" t="s">
         <v>187</v>
       </c>
-      <c r="C86" s="9" t="s">
+      <c r="C86" s="8" t="s">
         <v>187</v>
       </c>
       <c r="D86" s="6">
@@ -6953,7 +7096,7 @@
       <c r="G86" t="s">
         <v>353</v>
       </c>
-      <c r="H86" s="9" t="s">
+      <c r="H86" s="8" t="s">
         <v>186</v>
       </c>
       <c r="I86" t="str">
@@ -6968,7 +7111,7 @@
       <c r="B87" t="s">
         <v>189</v>
       </c>
-      <c r="C87" s="9" t="s">
+      <c r="C87" s="8" t="s">
         <v>189</v>
       </c>
       <c r="D87" s="6">
@@ -6981,7 +7124,7 @@
       <c r="G87" t="s">
         <v>353</v>
       </c>
-      <c r="H87" s="9" t="s">
+      <c r="H87" s="8" t="s">
         <v>188</v>
       </c>
       <c r="I87" t="str">
@@ -6996,7 +7139,7 @@
       <c r="B88" t="s">
         <v>191</v>
       </c>
-      <c r="C88" s="9" t="s">
+      <c r="C88" s="8" t="s">
         <v>191</v>
       </c>
       <c r="D88" s="6">
@@ -7009,7 +7152,7 @@
       <c r="G88" t="s">
         <v>353</v>
       </c>
-      <c r="H88" s="9" t="s">
+      <c r="H88" s="8" t="s">
         <v>190</v>
       </c>
       <c r="I88" t="str">
@@ -7024,7 +7167,7 @@
       <c r="B89" t="s">
         <v>193</v>
       </c>
-      <c r="C89" s="9" t="s">
+      <c r="C89" s="8" t="s">
         <v>193</v>
       </c>
       <c r="D89" s="6">
@@ -7037,7 +7180,7 @@
       <c r="G89" t="s">
         <v>353</v>
       </c>
-      <c r="H89" s="9" t="s">
+      <c r="H89" s="8" t="s">
         <v>192</v>
       </c>
       <c r="I89" t="str">
@@ -7052,7 +7195,7 @@
       <c r="B90" t="s">
         <v>196</v>
       </c>
-      <c r="C90" s="9" t="s">
+      <c r="C90" s="8" t="s">
         <v>196</v>
       </c>
       <c r="D90" s="6">
@@ -7065,7 +7208,7 @@
       <c r="G90" t="s">
         <v>353</v>
       </c>
-      <c r="H90" s="9" t="s">
+      <c r="H90" s="8" t="s">
         <v>194</v>
       </c>
       <c r="I90" t="str">
@@ -7080,7 +7223,7 @@
       <c r="B91" t="s">
         <v>199</v>
       </c>
-      <c r="C91" s="9" t="s">
+      <c r="C91" s="8" t="s">
         <v>199</v>
       </c>
       <c r="D91" s="6">
@@ -7093,7 +7236,7 @@
       <c r="G91" t="s">
         <v>353</v>
       </c>
-      <c r="H91" s="9" t="s">
+      <c r="H91" s="8" t="s">
         <v>197</v>
       </c>
       <c r="I91" t="str">
@@ -7108,7 +7251,7 @@
       <c r="B92" t="s">
         <v>201</v>
       </c>
-      <c r="C92" s="9" t="s">
+      <c r="C92" s="8" t="s">
         <v>201</v>
       </c>
       <c r="D92" s="6">
@@ -7121,7 +7264,7 @@
       <c r="G92" t="s">
         <v>353</v>
       </c>
-      <c r="H92" s="9" t="s">
+      <c r="H92" s="8" t="s">
         <v>200</v>
       </c>
       <c r="I92" t="str">
@@ -7136,7 +7279,7 @@
       <c r="B93" t="s">
         <v>203</v>
       </c>
-      <c r="C93" s="9" t="s">
+      <c r="C93" s="8" t="s">
         <v>203</v>
       </c>
       <c r="D93" s="6">
@@ -7149,7 +7292,7 @@
       <c r="G93" t="s">
         <v>353</v>
       </c>
-      <c r="H93" s="9" t="s">
+      <c r="H93" s="8" t="s">
         <v>202</v>
       </c>
       <c r="I93" t="str">
@@ -7164,7 +7307,7 @@
       <c r="B94" t="s">
         <v>205</v>
       </c>
-      <c r="C94" s="9" t="s">
+      <c r="C94" s="8" t="s">
         <v>205</v>
       </c>
       <c r="D94" s="6">
@@ -7177,7 +7320,7 @@
       <c r="G94" t="s">
         <v>353</v>
       </c>
-      <c r="H94" s="9" t="s">
+      <c r="H94" s="8" t="s">
         <v>204</v>
       </c>
       <c r="I94" t="str">
@@ -7192,7 +7335,7 @@
       <c r="B95" t="s">
         <v>207</v>
       </c>
-      <c r="C95" s="9" t="s">
+      <c r="C95" s="8" t="s">
         <v>207</v>
       </c>
       <c r="D95" s="6">
@@ -7205,7 +7348,7 @@
       <c r="G95" t="s">
         <v>353</v>
       </c>
-      <c r="H95" s="9" t="s">
+      <c r="H95" s="8" t="s">
         <v>206</v>
       </c>
       <c r="I95" t="str">
@@ -7220,7 +7363,7 @@
       <c r="B96" t="s">
         <v>209</v>
       </c>
-      <c r="C96" s="9" t="s">
+      <c r="C96" s="8" t="s">
         <v>209</v>
       </c>
       <c r="D96" s="6">
@@ -7233,7 +7376,7 @@
       <c r="G96" t="s">
         <v>353</v>
       </c>
-      <c r="H96" s="9" t="s">
+      <c r="H96" s="8" t="s">
         <v>208</v>
       </c>
       <c r="I96" t="str">
@@ -7248,7 +7391,7 @@
       <c r="B97" t="s">
         <v>212</v>
       </c>
-      <c r="C97" s="9" t="s">
+      <c r="C97" s="8" t="s">
         <v>212</v>
       </c>
       <c r="D97" s="6">
@@ -7261,7 +7404,7 @@
       <c r="G97" t="s">
         <v>353</v>
       </c>
-      <c r="H97" s="9" t="s">
+      <c r="H97" s="8" t="s">
         <v>210</v>
       </c>
       <c r="I97" t="str">
@@ -7276,7 +7419,7 @@
       <c r="B98" t="s">
         <v>214</v>
       </c>
-      <c r="C98" s="9" t="s">
+      <c r="C98" s="8" t="s">
         <v>214</v>
       </c>
       <c r="D98" s="6">
@@ -7289,7 +7432,7 @@
       <c r="G98" t="s">
         <v>353</v>
       </c>
-      <c r="H98" s="9" t="s">
+      <c r="H98" s="8" t="s">
         <v>213</v>
       </c>
       <c r="I98" t="str">
@@ -7304,7 +7447,7 @@
       <c r="B99" t="s">
         <v>216</v>
       </c>
-      <c r="C99" s="9" t="s">
+      <c r="C99" s="8" t="s">
         <v>216</v>
       </c>
       <c r="D99" s="6">
@@ -7317,7 +7460,7 @@
       <c r="G99" t="s">
         <v>353</v>
       </c>
-      <c r="H99" s="9" t="s">
+      <c r="H99" s="8" t="s">
         <v>215</v>
       </c>
       <c r="I99" t="str">
@@ -7332,7 +7475,7 @@
       <c r="B100" t="s">
         <v>218</v>
       </c>
-      <c r="C100" s="9" t="s">
+      <c r="C100" s="8" t="s">
         <v>218</v>
       </c>
       <c r="D100" s="6">
@@ -7345,7 +7488,7 @@
       <c r="G100" t="s">
         <v>353</v>
       </c>
-      <c r="H100" s="9" t="s">
+      <c r="H100" s="8" t="s">
         <v>217</v>
       </c>
       <c r="I100" t="str">
@@ -7360,7 +7503,7 @@
       <c r="B101" t="s">
         <v>220</v>
       </c>
-      <c r="C101" s="9" t="s">
+      <c r="C101" s="8" t="s">
         <v>220</v>
       </c>
       <c r="D101" s="6">
@@ -7373,7 +7516,7 @@
       <c r="G101" t="s">
         <v>353</v>
       </c>
-      <c r="H101" s="9" t="s">
+      <c r="H101" s="8" t="s">
         <v>219</v>
       </c>
       <c r="I101" t="str">
@@ -7388,7 +7531,7 @@
       <c r="B102" t="s">
         <v>222</v>
       </c>
-      <c r="C102" s="9" t="s">
+      <c r="C102" s="8" t="s">
         <v>222</v>
       </c>
       <c r="D102" s="6">
@@ -7401,7 +7544,7 @@
       <c r="G102" t="s">
         <v>353</v>
       </c>
-      <c r="H102" s="9" t="s">
+      <c r="H102" s="8" t="s">
         <v>355</v>
       </c>
       <c r="I102" t="str">
@@ -7416,7 +7559,7 @@
       <c r="B103" t="s">
         <v>224</v>
       </c>
-      <c r="C103" s="9" t="s">
+      <c r="C103" s="8" t="s">
         <v>224</v>
       </c>
       <c r="D103" s="6">
@@ -7429,7 +7572,7 @@
       <c r="G103" t="s">
         <v>353</v>
       </c>
-      <c r="H103" s="9" t="s">
+      <c r="H103" s="8" t="s">
         <v>223</v>
       </c>
       <c r="I103" t="str">
@@ -7444,7 +7587,7 @@
       <c r="B104" t="s">
         <v>226</v>
       </c>
-      <c r="C104" s="9" t="s">
+      <c r="C104" s="8" t="s">
         <v>226</v>
       </c>
       <c r="D104" s="6">
@@ -7457,7 +7600,7 @@
       <c r="G104" t="s">
         <v>353</v>
       </c>
-      <c r="H104" s="9" t="s">
+      <c r="H104" s="8" t="s">
         <v>225</v>
       </c>
       <c r="I104" t="str">
@@ -7472,7 +7615,7 @@
       <c r="B105" t="s">
         <v>228</v>
       </c>
-      <c r="C105" s="9" t="s">
+      <c r="C105" s="8" t="s">
         <v>228</v>
       </c>
       <c r="D105" s="6">
@@ -7485,7 +7628,7 @@
       <c r="G105" t="s">
         <v>353</v>
       </c>
-      <c r="H105" s="9" t="s">
+      <c r="H105" s="8" t="s">
         <v>227</v>
       </c>
       <c r="I105" t="str">
@@ -7500,7 +7643,7 @@
       <c r="B106" t="s">
         <v>230</v>
       </c>
-      <c r="C106" s="9" t="s">
+      <c r="C106" s="8" t="s">
         <v>230</v>
       </c>
       <c r="D106" s="6">
@@ -7513,7 +7656,7 @@
       <c r="G106" t="s">
         <v>353</v>
       </c>
-      <c r="H106" s="9" t="s">
+      <c r="H106" s="8" t="s">
         <v>229</v>
       </c>
       <c r="I106" t="str">
@@ -7528,7 +7671,7 @@
       <c r="B107" t="s">
         <v>232</v>
       </c>
-      <c r="C107" s="9" t="s">
+      <c r="C107" s="8" t="s">
         <v>232</v>
       </c>
       <c r="D107" s="6">
@@ -7541,7 +7684,7 @@
       <c r="G107" t="s">
         <v>353</v>
       </c>
-      <c r="H107" s="9" t="s">
+      <c r="H107" s="8" t="s">
         <v>231</v>
       </c>
       <c r="I107" t="str">
@@ -7556,7 +7699,7 @@
       <c r="B108" t="s">
         <v>234</v>
       </c>
-      <c r="C108" s="9" t="s">
+      <c r="C108" s="8" t="s">
         <v>234</v>
       </c>
       <c r="D108" s="6">
@@ -7569,7 +7712,7 @@
       <c r="G108" t="s">
         <v>353</v>
       </c>
-      <c r="H108" s="9" t="s">
+      <c r="H108" s="8" t="s">
         <v>233</v>
       </c>
       <c r="I108" t="str">
@@ -7584,7 +7727,7 @@
       <c r="B109" t="s">
         <v>236</v>
       </c>
-      <c r="C109" s="9" t="s">
+      <c r="C109" s="8" t="s">
         <v>236</v>
       </c>
       <c r="D109" s="6">
@@ -7597,7 +7740,7 @@
       <c r="G109" t="s">
         <v>353</v>
       </c>
-      <c r="H109" s="9" t="s">
+      <c r="H109" s="8" t="s">
         <v>235</v>
       </c>
       <c r="I109" t="str">
@@ -7612,7 +7755,7 @@
       <c r="B110" t="s">
         <v>238</v>
       </c>
-      <c r="C110" s="9" t="s">
+      <c r="C110" s="8" t="s">
         <v>238</v>
       </c>
       <c r="D110" s="6">
@@ -7625,7 +7768,7 @@
       <c r="G110" t="s">
         <v>353</v>
       </c>
-      <c r="H110" s="9" t="s">
+      <c r="H110" s="8" t="s">
         <v>237</v>
       </c>
       <c r="I110" t="str">
@@ -7640,7 +7783,7 @@
       <c r="B111" t="s">
         <v>240</v>
       </c>
-      <c r="C111" s="9" t="s">
+      <c r="C111" s="8" t="s">
         <v>240</v>
       </c>
       <c r="D111" s="6">
@@ -7653,7 +7796,7 @@
       <c r="G111" t="s">
         <v>353</v>
       </c>
-      <c r="H111" s="9" t="s">
+      <c r="H111" s="8" t="s">
         <v>239</v>
       </c>
       <c r="I111" t="str">
@@ -7681,10 +7824,10 @@
       <c r="G112" t="s">
         <v>353</v>
       </c>
-      <c r="H112" s="10" t="s">
+      <c r="H112" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="I112" s="11" t="str">
+      <c r="I112" s="10" t="str">
         <f t="shared" si="2"/>
         <v>Si</v>
       </c>
@@ -7696,7 +7839,7 @@
       <c r="B113" t="s">
         <v>244</v>
       </c>
-      <c r="C113" s="9" t="s">
+      <c r="C113" s="8" t="s">
         <v>244</v>
       </c>
       <c r="D113" s="6">
@@ -7709,7 +7852,7 @@
       <c r="G113" t="s">
         <v>353</v>
       </c>
-      <c r="H113" s="9" t="s">
+      <c r="H113" s="8" t="s">
         <v>243</v>
       </c>
       <c r="I113" t="str">
@@ -7724,7 +7867,7 @@
       <c r="B114" t="s">
         <v>246</v>
       </c>
-      <c r="C114" s="9" t="s">
+      <c r="C114" s="8" t="s">
         <v>246</v>
       </c>
       <c r="D114" s="6">
@@ -7737,7 +7880,7 @@
       <c r="G114" t="s">
         <v>353</v>
       </c>
-      <c r="H114" s="9" t="s">
+      <c r="H114" s="8" t="s">
         <v>245</v>
       </c>
       <c r="I114" t="str">
@@ -7752,7 +7895,7 @@
       <c r="B115" t="s">
         <v>248</v>
       </c>
-      <c r="C115" s="9" t="s">
+      <c r="C115" s="8" t="s">
         <v>248</v>
       </c>
       <c r="D115" s="6">
@@ -7765,7 +7908,7 @@
       <c r="G115" t="s">
         <v>353</v>
       </c>
-      <c r="H115" s="9" t="s">
+      <c r="H115" s="8" t="s">
         <v>247</v>
       </c>
       <c r="I115" t="str">
@@ -7780,7 +7923,7 @@
       <c r="B116" t="s">
         <v>250</v>
       </c>
-      <c r="C116" s="9" t="s">
+      <c r="C116" s="8" t="s">
         <v>250</v>
       </c>
       <c r="D116" s="6">
@@ -7793,7 +7936,7 @@
       <c r="G116" t="s">
         <v>353</v>
       </c>
-      <c r="H116" s="9" t="s">
+      <c r="H116" s="8" t="s">
         <v>249</v>
       </c>
       <c r="I116" t="str">
@@ -7808,7 +7951,7 @@
       <c r="B117" t="s">
         <v>252</v>
       </c>
-      <c r="C117" s="9" t="s">
+      <c r="C117" s="8" t="s">
         <v>252</v>
       </c>
       <c r="D117" s="6">
@@ -7821,7 +7964,7 @@
       <c r="G117" t="s">
         <v>353</v>
       </c>
-      <c r="H117" s="9" t="s">
+      <c r="H117" s="8" t="s">
         <v>251</v>
       </c>
       <c r="I117" t="str">
@@ -7836,7 +7979,7 @@
       <c r="B118" t="s">
         <v>254</v>
       </c>
-      <c r="C118" s="9" t="s">
+      <c r="C118" s="8" t="s">
         <v>254</v>
       </c>
       <c r="D118" s="6">
@@ -7849,7 +7992,7 @@
       <c r="G118" t="s">
         <v>353</v>
       </c>
-      <c r="H118" s="9" t="s">
+      <c r="H118" s="8" t="s">
         <v>253</v>
       </c>
       <c r="I118" t="str">
@@ -7864,7 +8007,7 @@
       <c r="B119" t="s">
         <v>256</v>
       </c>
-      <c r="C119" s="9" t="s">
+      <c r="C119" s="8" t="s">
         <v>256</v>
       </c>
       <c r="D119" s="6">
@@ -7877,7 +8020,7 @@
       <c r="G119" t="s">
         <v>353</v>
       </c>
-      <c r="H119" s="9" t="s">
+      <c r="H119" s="8" t="s">
         <v>255</v>
       </c>
       <c r="I119" t="str">
@@ -7892,7 +8035,7 @@
       <c r="B120" t="s">
         <v>258</v>
       </c>
-      <c r="C120" s="9" t="s">
+      <c r="C120" s="8" t="s">
         <v>258</v>
       </c>
       <c r="D120" s="6">
@@ -7905,7 +8048,7 @@
       <c r="G120" t="s">
         <v>353</v>
       </c>
-      <c r="H120" s="9" t="s">
+      <c r="H120" s="8" t="s">
         <v>257</v>
       </c>
       <c r="I120" t="str">
@@ -7920,7 +8063,7 @@
       <c r="B121" t="s">
         <v>260</v>
       </c>
-      <c r="C121" s="9" t="s">
+      <c r="C121" s="8" t="s">
         <v>260</v>
       </c>
       <c r="D121" s="6">
@@ -7933,7 +8076,7 @@
       <c r="G121" t="s">
         <v>353</v>
       </c>
-      <c r="H121" s="9" t="s">
+      <c r="H121" s="8" t="s">
         <v>259</v>
       </c>
       <c r="I121" t="str">
@@ -7948,7 +8091,7 @@
       <c r="B122" t="s">
         <v>262</v>
       </c>
-      <c r="C122" s="9" t="s">
+      <c r="C122" s="8" t="s">
         <v>262</v>
       </c>
       <c r="D122" s="6">
@@ -7961,7 +8104,7 @@
       <c r="G122" t="s">
         <v>353</v>
       </c>
-      <c r="H122" s="9" t="s">
+      <c r="H122" s="8" t="s">
         <v>261</v>
       </c>
       <c r="I122" t="str">
@@ -7976,7 +8119,7 @@
       <c r="B123" t="s">
         <v>264</v>
       </c>
-      <c r="C123" s="9" t="s">
+      <c r="C123" s="8" t="s">
         <v>264</v>
       </c>
       <c r="D123" s="6">
@@ -7989,7 +8132,7 @@
       <c r="G123" t="s">
         <v>353</v>
       </c>
-      <c r="H123" s="9" t="s">
+      <c r="H123" s="8" t="s">
         <v>263</v>
       </c>
       <c r="I123" t="str">
@@ -8004,7 +8147,7 @@
       <c r="B124" t="s">
         <v>266</v>
       </c>
-      <c r="C124" s="9" t="s">
+      <c r="C124" s="8" t="s">
         <v>266</v>
       </c>
       <c r="D124" s="6">
@@ -8017,7 +8160,7 @@
       <c r="G124" t="s">
         <v>353</v>
       </c>
-      <c r="H124" s="9" t="s">
+      <c r="H124" s="8" t="s">
         <v>265</v>
       </c>
       <c r="I124" t="str">
@@ -8032,7 +8175,7 @@
       <c r="B125" t="s">
         <v>268</v>
       </c>
-      <c r="C125" s="9" t="s">
+      <c r="C125" s="8" t="s">
         <v>268</v>
       </c>
       <c r="D125" s="6">
@@ -8045,7 +8188,7 @@
       <c r="G125" t="s">
         <v>353</v>
       </c>
-      <c r="H125" s="9" t="s">
+      <c r="H125" s="8" t="s">
         <v>267</v>
       </c>
       <c r="I125" t="str">
@@ -8060,7 +8203,7 @@
       <c r="B126" t="s">
         <v>270</v>
       </c>
-      <c r="C126" s="9" t="s">
+      <c r="C126" s="8" t="s">
         <v>270</v>
       </c>
       <c r="D126" s="6">
@@ -8073,7 +8216,7 @@
       <c r="G126" t="s">
         <v>353</v>
       </c>
-      <c r="H126" s="9" t="s">
+      <c r="H126" s="8" t="s">
         <v>269</v>
       </c>
       <c r="I126" t="str">
@@ -8088,7 +8231,7 @@
       <c r="B127" t="s">
         <v>272</v>
       </c>
-      <c r="C127" s="9" t="s">
+      <c r="C127" s="8" t="s">
         <v>272</v>
       </c>
       <c r="D127" s="6">
@@ -8101,7 +8244,7 @@
       <c r="G127" t="s">
         <v>353</v>
       </c>
-      <c r="H127" s="9" t="s">
+      <c r="H127" s="8" t="s">
         <v>271</v>
       </c>
       <c r="I127" t="str">
@@ -8116,7 +8259,7 @@
       <c r="B128" t="s">
         <v>274</v>
       </c>
-      <c r="C128" s="9" t="s">
+      <c r="C128" s="8" t="s">
         <v>274</v>
       </c>
       <c r="D128" s="6">
@@ -8129,7 +8272,7 @@
       <c r="G128" t="s">
         <v>353</v>
       </c>
-      <c r="H128" s="9" t="s">
+      <c r="H128" s="8" t="s">
         <v>273</v>
       </c>
       <c r="I128" t="str">
@@ -8144,7 +8287,7 @@
       <c r="B129" t="s">
         <v>276</v>
       </c>
-      <c r="C129" s="9" t="s">
+      <c r="C129" s="8" t="s">
         <v>276</v>
       </c>
       <c r="D129" s="6">
@@ -8157,7 +8300,7 @@
       <c r="G129" t="s">
         <v>353</v>
       </c>
-      <c r="H129" s="9" t="s">
+      <c r="H129" s="8" t="s">
         <v>275</v>
       </c>
       <c r="I129" t="str">
@@ -8172,7 +8315,7 @@
       <c r="B130" t="s">
         <v>278</v>
       </c>
-      <c r="C130" s="9" t="s">
+      <c r="C130" s="8" t="s">
         <v>278</v>
       </c>
       <c r="D130" s="6">
@@ -8185,7 +8328,7 @@
       <c r="G130" t="s">
         <v>353</v>
       </c>
-      <c r="H130" s="9" t="s">
+      <c r="H130" s="8" t="s">
         <v>277</v>
       </c>
       <c r="I130" t="str">
@@ -8200,7 +8343,7 @@
       <c r="B131" t="s">
         <v>280</v>
       </c>
-      <c r="C131" s="9" t="s">
+      <c r="C131" s="8" t="s">
         <v>280</v>
       </c>
       <c r="D131" s="6">
@@ -8213,7 +8356,7 @@
       <c r="G131" t="s">
         <v>353</v>
       </c>
-      <c r="H131" s="9" t="s">
+      <c r="H131" s="8" t="s">
         <v>279</v>
       </c>
       <c r="I131" t="str">
@@ -8228,7 +8371,7 @@
       <c r="B132" t="s">
         <v>282</v>
       </c>
-      <c r="C132" s="9" t="s">
+      <c r="C132" s="8" t="s">
         <v>282</v>
       </c>
       <c r="D132" s="6">
@@ -8241,7 +8384,7 @@
       <c r="G132" t="s">
         <v>353</v>
       </c>
-      <c r="H132" s="9" t="s">
+      <c r="H132" s="8" t="s">
         <v>281</v>
       </c>
       <c r="I132" t="str">
@@ -8256,7 +8399,7 @@
       <c r="B133" t="s">
         <v>284</v>
       </c>
-      <c r="C133" s="9" t="s">
+      <c r="C133" s="8" t="s">
         <v>284</v>
       </c>
       <c r="D133" s="6">
@@ -8269,7 +8412,7 @@
       <c r="G133" t="s">
         <v>353</v>
       </c>
-      <c r="H133" s="9" t="s">
+      <c r="H133" s="8" t="s">
         <v>283</v>
       </c>
       <c r="I133" t="str">
@@ -8297,10 +8440,10 @@
       <c r="G134" t="s">
         <v>353</v>
       </c>
-      <c r="H134" s="10" t="s">
+      <c r="H134" s="9" t="s">
         <v>285</v>
       </c>
-      <c r="I134" s="11" t="str">
+      <c r="I134" s="10" t="str">
         <f t="shared" ref="I134:I149" si="4">IF(E134=H134,"Si","No")</f>
         <v>Si</v>
       </c>
@@ -8312,7 +8455,7 @@
       <c r="B135" t="s">
         <v>289</v>
       </c>
-      <c r="C135" s="9" t="s">
+      <c r="C135" s="8" t="s">
         <v>289</v>
       </c>
       <c r="D135" s="6">
@@ -8325,7 +8468,7 @@
       <c r="G135" t="s">
         <v>353</v>
       </c>
-      <c r="H135" s="9" t="s">
+      <c r="H135" s="8" t="s">
         <v>287</v>
       </c>
       <c r="I135" t="str">
@@ -8340,7 +8483,7 @@
       <c r="B136" t="s">
         <v>291</v>
       </c>
-      <c r="C136" s="9" t="s">
+      <c r="C136" s="8" t="s">
         <v>291</v>
       </c>
       <c r="D136" s="6">
@@ -8353,7 +8496,7 @@
       <c r="G136" t="s">
         <v>353</v>
       </c>
-      <c r="H136" s="9" t="s">
+      <c r="H136" s="8" t="s">
         <v>290</v>
       </c>
       <c r="I136" t="str">
@@ -8368,7 +8511,7 @@
       <c r="B137" t="s">
         <v>293</v>
       </c>
-      <c r="C137" s="9" t="s">
+      <c r="C137" s="8" t="s">
         <v>293</v>
       </c>
       <c r="D137" s="6">
@@ -8381,7 +8524,7 @@
       <c r="G137" t="s">
         <v>353</v>
       </c>
-      <c r="H137" s="9" t="s">
+      <c r="H137" s="8" t="s">
         <v>292</v>
       </c>
       <c r="I137" t="str">
@@ -8396,7 +8539,7 @@
       <c r="B138" t="s">
         <v>295</v>
       </c>
-      <c r="C138" s="9" t="s">
+      <c r="C138" s="8" t="s">
         <v>295</v>
       </c>
       <c r="D138" s="6">
@@ -8409,7 +8552,7 @@
       <c r="G138" t="s">
         <v>353</v>
       </c>
-      <c r="H138" s="9" t="s">
+      <c r="H138" s="8" t="s">
         <v>294</v>
       </c>
       <c r="I138" t="str">
@@ -8424,7 +8567,7 @@
       <c r="B139" t="s">
         <v>298</v>
       </c>
-      <c r="C139" s="9" t="s">
+      <c r="C139" s="8" t="s">
         <v>298</v>
       </c>
       <c r="D139" s="6">
@@ -8437,7 +8580,7 @@
       <c r="G139" t="s">
         <v>353</v>
       </c>
-      <c r="H139" s="9" t="s">
+      <c r="H139" s="8" t="s">
         <v>296</v>
       </c>
       <c r="I139" t="str">
@@ -8452,7 +8595,7 @@
       <c r="B140" t="s">
         <v>300</v>
       </c>
-      <c r="C140" s="9" t="s">
+      <c r="C140" s="8" t="s">
         <v>300</v>
       </c>
       <c r="D140" s="6">
@@ -8465,7 +8608,7 @@
       <c r="G140" t="s">
         <v>353</v>
       </c>
-      <c r="H140" s="9" t="s">
+      <c r="H140" s="8" t="s">
         <v>299</v>
       </c>
       <c r="I140" t="str">
@@ -8480,7 +8623,7 @@
       <c r="B141" t="s">
         <v>302</v>
       </c>
-      <c r="C141" s="9" t="s">
+      <c r="C141" s="8" t="s">
         <v>302</v>
       </c>
       <c r="D141" s="6">
@@ -8493,7 +8636,7 @@
       <c r="G141" t="s">
         <v>353</v>
       </c>
-      <c r="H141" s="9" t="s">
+      <c r="H141" s="8" t="s">
         <v>301</v>
       </c>
       <c r="I141" t="str">
@@ -8508,7 +8651,7 @@
       <c r="B142" t="s">
         <v>304</v>
       </c>
-      <c r="C142" s="9" t="s">
+      <c r="C142" s="8" t="s">
         <v>304</v>
       </c>
       <c r="D142" s="6">
@@ -8521,7 +8664,7 @@
       <c r="G142" t="s">
         <v>353</v>
       </c>
-      <c r="H142" s="9" t="s">
+      <c r="H142" s="8" t="s">
         <v>303</v>
       </c>
       <c r="I142" t="str">
@@ -8536,7 +8679,7 @@
       <c r="B143" t="s">
         <v>306</v>
       </c>
-      <c r="C143" s="9" t="s">
+      <c r="C143" s="8" t="s">
         <v>306</v>
       </c>
       <c r="D143" s="6">
@@ -8549,7 +8692,7 @@
       <c r="G143" t="s">
         <v>353</v>
       </c>
-      <c r="H143" s="9" t="s">
+      <c r="H143" s="8" t="s">
         <v>305</v>
       </c>
       <c r="I143" t="str">
@@ -8564,7 +8707,7 @@
       <c r="B144" t="s">
         <v>308</v>
       </c>
-      <c r="C144" s="9" t="s">
+      <c r="C144" s="8" t="s">
         <v>308</v>
       </c>
       <c r="D144" s="6">
@@ -8577,7 +8720,7 @@
       <c r="G144" t="s">
         <v>353</v>
       </c>
-      <c r="H144" s="9" t="s">
+      <c r="H144" s="8" t="s">
         <v>307</v>
       </c>
       <c r="I144" t="str">
@@ -8592,7 +8735,7 @@
       <c r="B145" t="s">
         <v>310</v>
       </c>
-      <c r="C145" s="9" t="s">
+      <c r="C145" s="8" t="s">
         <v>310</v>
       </c>
       <c r="D145" s="6">
@@ -8605,7 +8748,7 @@
       <c r="G145" t="s">
         <v>353</v>
       </c>
-      <c r="H145" s="9" t="s">
+      <c r="H145" s="8" t="s">
         <v>309</v>
       </c>
       <c r="I145" t="str">
@@ -8620,7 +8763,7 @@
       <c r="B146" t="s">
         <v>313</v>
       </c>
-      <c r="C146" s="9" t="s">
+      <c r="C146" s="8" t="s">
         <v>313</v>
       </c>
       <c r="D146" s="6">
@@ -8633,7 +8776,7 @@
       <c r="G146" t="s">
         <v>353</v>
       </c>
-      <c r="H146" s="9" t="s">
+      <c r="H146" s="8" t="s">
         <v>311</v>
       </c>
       <c r="I146" t="str">
@@ -8648,7 +8791,7 @@
       <c r="B147" t="s">
         <v>315</v>
       </c>
-      <c r="C147" s="9" t="s">
+      <c r="C147" s="8" t="s">
         <v>315</v>
       </c>
       <c r="D147" s="6">
@@ -8661,7 +8804,7 @@
       <c r="G147" t="s">
         <v>353</v>
       </c>
-      <c r="H147" s="9" t="s">
+      <c r="H147" s="8" t="s">
         <v>314</v>
       </c>
       <c r="I147" t="str">
@@ -8676,7 +8819,7 @@
       <c r="B148" t="s">
         <v>317</v>
       </c>
-      <c r="C148" s="9" t="s">
+      <c r="C148" s="8" t="s">
         <v>317</v>
       </c>
       <c r="D148" s="6">
@@ -8689,7 +8832,7 @@
       <c r="G148" t="s">
         <v>353</v>
       </c>
-      <c r="H148" s="9" t="s">
+      <c r="H148" s="8" t="s">
         <v>316</v>
       </c>
       <c r="I148" t="str">
@@ -8704,7 +8847,7 @@
       <c r="B149" t="s">
         <v>319</v>
       </c>
-      <c r="C149" s="9" t="s">
+      <c r="C149" s="8" t="s">
         <v>319</v>
       </c>
       <c r="D149" s="6">
@@ -8717,7 +8860,7 @@
       <c r="G149" t="s">
         <v>353</v>
       </c>
-      <c r="H149" s="9" t="s">
+      <c r="H149" s="8" t="s">
         <v>318</v>
       </c>
       <c r="I149" t="str">
@@ -8732,7 +8875,7 @@
       <c r="B150" t="s">
         <v>321</v>
       </c>
-      <c r="C150" s="9" t="s">
+      <c r="C150" s="8" t="s">
         <v>321</v>
       </c>
       <c r="D150" s="6">
@@ -8745,7 +8888,7 @@
       <c r="G150" t="s">
         <v>353</v>
       </c>
-      <c r="H150" s="9" t="s">
+      <c r="H150" s="8" t="s">
         <v>320</v>
       </c>
       <c r="I150" t="str">
@@ -8760,7 +8903,7 @@
       <c r="B151" t="s">
         <v>336</v>
       </c>
-      <c r="C151" s="9" t="s">
+      <c r="C151" s="8" t="s">
         <v>336</v>
       </c>
       <c r="D151" s="6">
@@ -8781,7 +8924,7 @@
       <c r="B152" t="s">
         <v>337</v>
       </c>
-      <c r="C152" s="9" t="s">
+      <c r="C152" s="8" t="s">
         <v>337</v>
       </c>
       <c r="D152" s="6">
@@ -8802,7 +8945,7 @@
       <c r="B153" t="s">
         <v>325</v>
       </c>
-      <c r="C153" s="9" t="s">
+      <c r="C153" s="8" t="s">
         <v>356</v>
       </c>
       <c r="D153" s="1" t="s">
@@ -8822,7 +8965,7 @@
       <c r="B154" t="s">
         <v>326</v>
       </c>
-      <c r="C154" s="9" t="s">
+      <c r="C154" s="8" t="s">
         <v>357</v>
       </c>
       <c r="D154" s="1" t="s">
@@ -8842,7 +8985,7 @@
       <c r="B155" t="s">
         <v>327</v>
       </c>
-      <c r="C155" s="9" t="s">
+      <c r="C155" s="8" t="s">
         <v>358</v>
       </c>
       <c r="D155" s="1" t="s">
@@ -8862,7 +9005,7 @@
       <c r="B156" t="s">
         <v>328</v>
       </c>
-      <c r="C156" s="9" t="s">
+      <c r="C156" s="8" t="s">
         <v>359</v>
       </c>
       <c r="D156" s="1" t="s">
@@ -8882,7 +9025,7 @@
       <c r="B157" t="s">
         <v>329</v>
       </c>
-      <c r="C157" s="9" t="s">
+      <c r="C157" s="8" t="s">
         <v>360</v>
       </c>
       <c r="D157" s="1" t="s">
@@ -8902,7 +9045,7 @@
       <c r="B158" t="s">
         <v>330</v>
       </c>
-      <c r="C158" s="9" t="s">
+      <c r="C158" s="8" t="s">
         <v>361</v>
       </c>
       <c r="D158" s="1" t="s">
@@ -8922,7 +9065,7 @@
       <c r="B159" t="s">
         <v>331</v>
       </c>
-      <c r="C159" s="9" t="s">
+      <c r="C159" s="8" t="s">
         <v>362</v>
       </c>
       <c r="D159" s="1" t="s">
@@ -8942,7 +9085,7 @@
       <c r="B160" t="s">
         <v>332</v>
       </c>
-      <c r="C160" s="9" t="s">
+      <c r="C160" s="8" t="s">
         <v>363</v>
       </c>
       <c r="D160" s="1" t="s">
@@ -8959,4 +9102,674 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9DD7D967-4348-4E8F-A6E6-EFD3CF851029}">
+  <dimension ref="A1:D149"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="32.7109375" customWidth="1"/>
+    <col min="2" max="2" width="50.28515625" customWidth="1"/>
+    <col min="3" max="3" width="32.7109375" customWidth="1"/>
+    <col min="4" max="4" width="37" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4">
+      <c r="A1" s="11" t="s">
+        <v>364</v>
+      </c>
+      <c r="B1" s="11"/>
+      <c r="C1" s="11" t="s">
+        <v>388</v>
+      </c>
+      <c r="D1" s="11"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="12" t="s">
+        <v>365</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>366</v>
+      </c>
+      <c r="C3" s="12" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="12" t="s">
+        <v>368</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="12" t="s">
+        <v>369</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="12" t="s">
+        <v>370</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="A8" s="12" t="s">
+        <v>371</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="12" t="s">
+        <v>372</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
+      <c r="A10" s="12" t="s">
+        <v>373</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
+      <c r="A11" s="12" t="s">
+        <v>374</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
+      <c r="A12" s="12" t="s">
+        <v>375</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
+      <c r="A13" s="12" t="s">
+        <v>376</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="12" t="s">
+        <v>377</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
+      <c r="A15" s="12" t="s">
+        <v>378</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
+      <c r="A16" s="12" t="s">
+        <v>379</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="12" t="s">
+        <v>380</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>403</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="12" t="s">
+        <v>381</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" s="12" t="s">
+        <v>382</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" s="12" t="s">
+        <v>383</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" s="12" t="s">
+        <v>384</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" s="12" t="s">
+        <v>385</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" s="12" t="s">
+        <v>386</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" s="12" t="s">
+        <v>387</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="C26" s="12"/>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="C27" s="12"/>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="C28" s="12"/>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="C29" s="12"/>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="C30" s="12"/>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="C31" s="12"/>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="C32" s="12"/>
+    </row>
+    <row r="33" spans="3:3">
+      <c r="C33" s="12"/>
+    </row>
+    <row r="34" spans="3:3">
+      <c r="C34" s="12"/>
+    </row>
+    <row r="35" spans="3:3">
+      <c r="C35" s="12"/>
+    </row>
+    <row r="36" spans="3:3">
+      <c r="C36" s="12"/>
+    </row>
+    <row r="37" spans="3:3">
+      <c r="C37" s="12"/>
+    </row>
+    <row r="38" spans="3:3">
+      <c r="C38" s="12"/>
+    </row>
+    <row r="39" spans="3:3">
+      <c r="C39" s="12"/>
+    </row>
+    <row r="40" spans="3:3">
+      <c r="C40" s="12"/>
+    </row>
+    <row r="41" spans="3:3">
+      <c r="C41" s="12"/>
+    </row>
+    <row r="42" spans="3:3">
+      <c r="C42" s="12"/>
+    </row>
+    <row r="43" spans="3:3">
+      <c r="C43" s="12"/>
+    </row>
+    <row r="44" spans="3:3">
+      <c r="C44" s="12"/>
+    </row>
+    <row r="45" spans="3:3">
+      <c r="C45" s="12"/>
+    </row>
+    <row r="46" spans="3:3">
+      <c r="C46" s="12"/>
+    </row>
+    <row r="47" spans="3:3">
+      <c r="C47" s="12"/>
+    </row>
+    <row r="48" spans="3:3">
+      <c r="C48" s="12"/>
+    </row>
+    <row r="49" spans="3:3">
+      <c r="C49" s="12"/>
+    </row>
+    <row r="50" spans="3:3">
+      <c r="C50" s="12"/>
+    </row>
+    <row r="51" spans="3:3">
+      <c r="C51" s="12"/>
+    </row>
+    <row r="52" spans="3:3">
+      <c r="C52" s="12"/>
+    </row>
+    <row r="53" spans="3:3">
+      <c r="C53" s="12"/>
+    </row>
+    <row r="54" spans="3:3">
+      <c r="C54" s="12"/>
+    </row>
+    <row r="55" spans="3:3">
+      <c r="C55" s="12"/>
+    </row>
+    <row r="56" spans="3:3">
+      <c r="C56" s="12"/>
+    </row>
+    <row r="57" spans="3:3">
+      <c r="C57" s="12"/>
+    </row>
+    <row r="58" spans="3:3">
+      <c r="C58" s="12"/>
+    </row>
+    <row r="59" spans="3:3">
+      <c r="C59" s="12"/>
+    </row>
+    <row r="60" spans="3:3">
+      <c r="C60" s="12"/>
+    </row>
+    <row r="61" spans="3:3">
+      <c r="C61" s="12"/>
+    </row>
+    <row r="62" spans="3:3">
+      <c r="C62" s="12"/>
+    </row>
+    <row r="63" spans="3:3">
+      <c r="C63" s="12"/>
+    </row>
+    <row r="64" spans="3:3">
+      <c r="C64" s="12"/>
+    </row>
+    <row r="65" spans="3:3">
+      <c r="C65" s="12"/>
+    </row>
+    <row r="66" spans="3:3">
+      <c r="C66" s="12"/>
+    </row>
+    <row r="67" spans="3:3">
+      <c r="C67" s="12"/>
+    </row>
+    <row r="68" spans="3:3">
+      <c r="C68" s="12"/>
+    </row>
+    <row r="69" spans="3:3">
+      <c r="C69" s="12"/>
+    </row>
+    <row r="70" spans="3:3">
+      <c r="C70" s="12"/>
+    </row>
+    <row r="71" spans="3:3">
+      <c r="C71" s="12"/>
+    </row>
+    <row r="72" spans="3:3">
+      <c r="C72" s="12"/>
+    </row>
+    <row r="73" spans="3:3">
+      <c r="C73" s="12"/>
+    </row>
+    <row r="74" spans="3:3">
+      <c r="C74" s="12"/>
+    </row>
+    <row r="75" spans="3:3">
+      <c r="C75" s="12"/>
+    </row>
+    <row r="76" spans="3:3">
+      <c r="C76" s="12"/>
+    </row>
+    <row r="77" spans="3:3">
+      <c r="C77" s="12"/>
+    </row>
+    <row r="78" spans="3:3">
+      <c r="C78" s="12"/>
+    </row>
+    <row r="79" spans="3:3">
+      <c r="C79" s="12"/>
+    </row>
+    <row r="80" spans="3:3">
+      <c r="C80" s="12"/>
+    </row>
+    <row r="81" spans="3:3">
+      <c r="C81" s="12"/>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" s="12"/>
+    </row>
+    <row r="83" spans="3:3">
+      <c r="C83" s="12"/>
+    </row>
+    <row r="84" spans="3:3">
+      <c r="C84" s="12"/>
+    </row>
+    <row r="85" spans="3:3">
+      <c r="C85" s="12"/>
+    </row>
+    <row r="86" spans="3:3">
+      <c r="C86" s="12"/>
+    </row>
+    <row r="87" spans="3:3">
+      <c r="C87" s="12"/>
+    </row>
+    <row r="88" spans="3:3">
+      <c r="C88" s="12"/>
+    </row>
+    <row r="89" spans="3:3">
+      <c r="C89" s="12"/>
+    </row>
+    <row r="90" spans="3:3">
+      <c r="C90" s="12"/>
+    </row>
+    <row r="91" spans="3:3">
+      <c r="C91" s="12"/>
+    </row>
+    <row r="92" spans="3:3">
+      <c r="C92" s="12"/>
+    </row>
+    <row r="93" spans="3:3">
+      <c r="C93" s="12"/>
+    </row>
+    <row r="94" spans="3:3">
+      <c r="C94" s="12"/>
+    </row>
+    <row r="95" spans="3:3">
+      <c r="C95" s="12"/>
+    </row>
+    <row r="96" spans="3:3">
+      <c r="C96" s="12"/>
+    </row>
+    <row r="97" spans="3:3">
+      <c r="C97" s="12"/>
+    </row>
+    <row r="98" spans="3:3">
+      <c r="C98" s="12"/>
+    </row>
+    <row r="99" spans="3:3">
+      <c r="C99" s="12"/>
+    </row>
+    <row r="100" spans="3:3">
+      <c r="C100" s="12"/>
+    </row>
+    <row r="101" spans="3:3">
+      <c r="C101" s="12"/>
+    </row>
+    <row r="102" spans="3:3">
+      <c r="C102" s="12"/>
+    </row>
+    <row r="103" spans="3:3">
+      <c r="C103" s="12"/>
+    </row>
+    <row r="104" spans="3:3">
+      <c r="C104" s="12"/>
+    </row>
+    <row r="105" spans="3:3">
+      <c r="C105" s="12"/>
+    </row>
+    <row r="106" spans="3:3">
+      <c r="C106" s="12"/>
+    </row>
+    <row r="107" spans="3:3">
+      <c r="C107" s="12"/>
+    </row>
+    <row r="108" spans="3:3">
+      <c r="C108" s="12"/>
+    </row>
+    <row r="109" spans="3:3">
+      <c r="C109" s="12"/>
+    </row>
+    <row r="110" spans="3:3">
+      <c r="C110" s="12"/>
+    </row>
+    <row r="111" spans="3:3">
+      <c r="C111" s="12"/>
+    </row>
+    <row r="112" spans="3:3">
+      <c r="C112" s="12"/>
+    </row>
+    <row r="113" spans="3:3">
+      <c r="C113" s="12"/>
+    </row>
+    <row r="114" spans="3:3">
+      <c r="C114" s="12"/>
+    </row>
+    <row r="115" spans="3:3">
+      <c r="C115" s="12"/>
+    </row>
+    <row r="116" spans="3:3">
+      <c r="C116" s="12"/>
+    </row>
+    <row r="117" spans="3:3">
+      <c r="C117" s="12"/>
+    </row>
+    <row r="118" spans="3:3">
+      <c r="C118" s="12"/>
+    </row>
+    <row r="119" spans="3:3">
+      <c r="C119" s="12"/>
+    </row>
+    <row r="120" spans="3:3">
+      <c r="C120" s="12"/>
+    </row>
+    <row r="121" spans="3:3">
+      <c r="C121" s="12"/>
+    </row>
+    <row r="122" spans="3:3">
+      <c r="C122" s="12"/>
+    </row>
+    <row r="123" spans="3:3">
+      <c r="C123" s="12"/>
+    </row>
+    <row r="124" spans="3:3">
+      <c r="C124" s="12"/>
+    </row>
+    <row r="125" spans="3:3">
+      <c r="C125" s="12"/>
+    </row>
+    <row r="126" spans="3:3">
+      <c r="C126" s="12"/>
+    </row>
+    <row r="127" spans="3:3">
+      <c r="C127" s="12"/>
+    </row>
+    <row r="128" spans="3:3">
+      <c r="C128" s="12"/>
+    </row>
+    <row r="129" spans="3:3">
+      <c r="C129" s="12"/>
+    </row>
+    <row r="130" spans="3:3">
+      <c r="C130" s="12"/>
+    </row>
+    <row r="131" spans="3:3">
+      <c r="C131" s="12"/>
+    </row>
+    <row r="132" spans="3:3">
+      <c r="C132" s="12"/>
+    </row>
+    <row r="133" spans="3:3">
+      <c r="C133" s="12"/>
+    </row>
+    <row r="134" spans="3:3">
+      <c r="C134" s="12"/>
+    </row>
+    <row r="135" spans="3:3">
+      <c r="C135" s="12"/>
+    </row>
+    <row r="136" spans="3:3">
+      <c r="C136" s="12"/>
+    </row>
+    <row r="137" spans="3:3">
+      <c r="C137" s="12"/>
+    </row>
+    <row r="138" spans="3:3">
+      <c r="C138" s="12"/>
+    </row>
+    <row r="139" spans="3:3">
+      <c r="C139" s="12"/>
+    </row>
+    <row r="140" spans="3:3">
+      <c r="C140" s="12"/>
+    </row>
+    <row r="141" spans="3:3">
+      <c r="C141" s="12"/>
+    </row>
+    <row r="142" spans="3:3">
+      <c r="C142" s="12"/>
+    </row>
+    <row r="143" spans="3:3">
+      <c r="C143" s="12"/>
+    </row>
+    <row r="144" spans="3:3">
+      <c r="C144" s="12"/>
+    </row>
+    <row r="145" spans="3:3">
+      <c r="C145" s="12"/>
+    </row>
+    <row r="146" spans="3:3">
+      <c r="C146" s="12"/>
+    </row>
+    <row r="147" spans="3:3">
+      <c r="C147" s="12"/>
+    </row>
+    <row r="148" spans="3:3">
+      <c r="C148" s="12"/>
+    </row>
+    <row r="149" spans="3:3">
+      <c r="C149" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="C1:D1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>